<commit_message>
[S6] feat: tracker rules (Financials D/E skip, SIMULATED labels, Makefile), final deliverables
</commit_message>
<xml_diff>
--- a/output/screener_output.xlsx
+++ b/output/screener_output.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z21"/>
+  <dimension ref="A1:Z23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1362,17 +1362,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Infosys Ltd</t>
+          <t>ICICI Bank Ltd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1381,84 +1381,86 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>61.6</v>
+        <v>61.8</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>29.79</v>
+        <v>17.99</v>
       </c>
       <c r="H11" t="n">
-        <v>32.91</v>
+        <v>5.12</v>
       </c>
       <c r="I11" t="n">
-        <v>17.08</v>
+        <v>28.89</v>
       </c>
       <c r="J11" t="n">
-        <v>23.7</v>
+        <v>62.41</v>
       </c>
       <c r="K11" t="n">
-        <v>0.09</v>
+        <v>6.45</v>
       </c>
       <c r="L11" t="n">
-        <v>87.52</v>
+        <v>1.3</v>
       </c>
       <c r="M11" t="n">
-        <v>20117</v>
+        <v>12547</v>
       </c>
       <c r="N11" t="n">
-        <v>13.09</v>
+        <v>7.87</v>
       </c>
       <c r="O11" t="n">
-        <v>1.81</v>
+        <v>0.95</v>
       </c>
       <c r="P11" t="n">
-        <v>15.22</v>
+        <v>21.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>13.2</v>
+        <v>17.25</v>
       </c>
       <c r="R11" t="n">
-        <v>11.24</v>
+        <v>51.95</v>
       </c>
       <c r="S11" t="n">
-        <v>12.47</v>
+        <v>55.18</v>
       </c>
       <c r="T11" t="n">
-        <v>0.96</v>
+        <v>3.41</v>
       </c>
       <c r="U11" t="n">
-        <v>35.99</v>
+        <v>25.76</v>
       </c>
       <c r="V11" t="n">
-        <v>8.970000000000001</v>
+        <v>6.2</v>
       </c>
       <c r="W11" t="n">
-        <v>36.7</v>
+        <v>38.28</v>
       </c>
       <c r="X11" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="Y11" t="inlineStr"/>
+        <v>3.43</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>16</v>
+      </c>
       <c r="Z11" t="n">
-        <v>153670</v>
+        <v>159516</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ATGL</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Adani Total Gas Ltd</t>
+          <t>Infosys Ltd</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1467,86 +1469,84 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>61.1</v>
+        <v>61.6</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>18.66</v>
+        <v>29.79</v>
       </c>
       <c r="H12" t="n">
-        <v>18.42</v>
+        <v>32.91</v>
       </c>
       <c r="I12" t="n">
-        <v>14.93</v>
+        <v>17.08</v>
       </c>
       <c r="J12" t="n">
-        <v>24.67</v>
+        <v>23.7</v>
       </c>
       <c r="K12" t="n">
-        <v>0.43</v>
+        <v>0.09</v>
       </c>
       <c r="L12" t="n">
-        <v>10.5</v>
+        <v>87.52</v>
       </c>
       <c r="M12" t="n">
-        <v>203</v>
+        <v>20117</v>
       </c>
       <c r="N12" t="n">
-        <v>4.54</v>
+        <v>13.09</v>
       </c>
       <c r="O12" t="n">
-        <v>0.01</v>
+        <v>1.81</v>
       </c>
       <c r="P12" t="n">
-        <v>38.18</v>
+        <v>15.22</v>
       </c>
       <c r="Q12" t="n">
-        <v>21.09</v>
+        <v>13.2</v>
       </c>
       <c r="R12" t="n">
-        <v>23.88</v>
+        <v>11.24</v>
       </c>
       <c r="S12" t="n">
-        <v>24.57</v>
+        <v>12.47</v>
       </c>
       <c r="T12" t="n">
-        <v>1.43</v>
+        <v>0.96</v>
       </c>
       <c r="U12" t="n">
-        <v>56.96</v>
+        <v>35.99</v>
       </c>
       <c r="V12" t="n">
-        <v>5.76</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="W12" t="n">
-        <v>28.93</v>
+        <v>36.7</v>
       </c>
       <c r="X12" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>4</v>
-      </c>
+        <v>4.1</v>
+      </c>
+      <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="n">
-        <v>4475</v>
+        <v>153670</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>ATGL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sun Pharmaceuticals Industries Ltd</t>
+          <t>Adani Total Gas Ltd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1555,86 +1555,86 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>60.9</v>
+        <v>61.1</v>
       </c>
       <c r="F13" t="n">
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>15.09</v>
+        <v>18.66</v>
       </c>
       <c r="H13" t="n">
-        <v>15.63</v>
+        <v>18.42</v>
       </c>
       <c r="I13" t="n">
-        <v>19.82</v>
+        <v>14.93</v>
       </c>
       <c r="J13" t="n">
-        <v>26.84</v>
+        <v>24.67</v>
       </c>
       <c r="K13" t="n">
-        <v>0.05</v>
+        <v>0.43</v>
       </c>
       <c r="L13" t="n">
-        <v>58.33</v>
+        <v>10.5</v>
       </c>
       <c r="M13" t="n">
-        <v>11372</v>
+        <v>203</v>
       </c>
       <c r="N13" t="n">
-        <v>23.45</v>
+        <v>4.54</v>
       </c>
       <c r="O13" t="n">
-        <v>0.85</v>
+        <v>0.01</v>
       </c>
       <c r="P13" t="n">
-        <v>13.13</v>
+        <v>38.18</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.78</v>
+        <v>21.09</v>
       </c>
       <c r="R13" t="n">
-        <v>24.54</v>
+        <v>23.88</v>
       </c>
       <c r="S13" t="n">
-        <v>29.46</v>
+        <v>24.57</v>
       </c>
       <c r="T13" t="n">
-        <v>1.26</v>
+        <v>1.43</v>
       </c>
       <c r="U13" t="n">
-        <v>37.9</v>
+        <v>56.96</v>
       </c>
       <c r="V13" t="n">
-        <v>6.71</v>
+        <v>5.76</v>
       </c>
       <c r="W13" t="n">
-        <v>21.41</v>
+        <v>28.93</v>
       </c>
       <c r="X13" t="n">
-        <v>3.88</v>
+        <v>0.51</v>
       </c>
       <c r="Y13" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="Z13" t="n">
-        <v>48497</v>
+        <v>4475</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HCL Technologies Ltd</t>
+          <t>Sun Pharmaceuticals Industries Ltd</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1643,86 +1643,86 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>57.7</v>
+        <v>60.9</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>23.01</v>
+        <v>15.09</v>
       </c>
       <c r="H14" t="n">
-        <v>27.05</v>
+        <v>15.63</v>
       </c>
       <c r="I14" t="n">
-        <v>14.29</v>
+        <v>19.82</v>
       </c>
       <c r="J14" t="n">
-        <v>22.02</v>
+        <v>26.84</v>
       </c>
       <c r="K14" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
       <c r="L14" t="n">
-        <v>46.46</v>
+        <v>58.33</v>
       </c>
       <c r="M14" t="n">
-        <v>15840</v>
+        <v>11372</v>
       </c>
       <c r="N14" t="n">
-        <v>14.41</v>
+        <v>23.45</v>
       </c>
       <c r="O14" t="n">
-        <v>3.84</v>
+        <v>0.85</v>
       </c>
       <c r="P14" t="n">
-        <v>13.4</v>
+        <v>13.13</v>
       </c>
       <c r="Q14" t="n">
-        <v>12.71</v>
+        <v>10.78</v>
       </c>
       <c r="R14" t="n">
-        <v>9.19</v>
+        <v>24.54</v>
       </c>
       <c r="S14" t="n">
-        <v>9.41</v>
+        <v>29.46</v>
       </c>
       <c r="T14" t="n">
-        <v>1.43</v>
+        <v>1.26</v>
       </c>
       <c r="U14" t="n">
-        <v>63.63</v>
+        <v>37.9</v>
       </c>
       <c r="V14" t="n">
-        <v>5.44</v>
+        <v>6.71</v>
       </c>
       <c r="W14" t="n">
-        <v>31.21</v>
+        <v>21.41</v>
       </c>
       <c r="X14" t="n">
-        <v>1.99</v>
+        <v>3.88</v>
       </c>
       <c r="Y14" t="n">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="Z14" t="n">
-        <v>109913</v>
+        <v>48497</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dr Reddys Laboratories Ltd</t>
+          <t>HCL Technologies Ltd</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1731,86 +1731,86 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>57.2</v>
+        <v>57.7</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>19.74</v>
+        <v>23.01</v>
       </c>
       <c r="H15" t="n">
-        <v>21.36</v>
+        <v>27.05</v>
       </c>
       <c r="I15" t="n">
-        <v>19.91</v>
+        <v>14.29</v>
       </c>
       <c r="J15" t="n">
-        <v>28.32</v>
+        <v>22.02</v>
       </c>
       <c r="K15" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="L15" t="n">
-        <v>51.71</v>
+        <v>46.46</v>
       </c>
       <c r="M15" t="n">
-        <v>509</v>
+        <v>15840</v>
       </c>
       <c r="N15" t="n">
-        <v>1.82</v>
+        <v>14.41</v>
       </c>
       <c r="O15" t="n">
-        <v>0.02</v>
+        <v>3.84</v>
       </c>
       <c r="P15" t="n">
-        <v>13.72</v>
+        <v>13.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>12.64</v>
+        <v>12.71</v>
       </c>
       <c r="R15" t="n">
-        <v>23.39</v>
+        <v>9.19</v>
       </c>
       <c r="S15" t="n">
-        <v>23.84</v>
+        <v>9.41</v>
       </c>
       <c r="T15" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.43</v>
       </c>
       <c r="U15" t="n">
-        <v>11.73</v>
+        <v>63.63</v>
       </c>
       <c r="V15" t="n">
-        <v>10.19</v>
+        <v>5.44</v>
       </c>
       <c r="W15" t="n">
-        <v>14.56</v>
+        <v>31.21</v>
       </c>
       <c r="X15" t="n">
-        <v>0.09</v>
+        <v>1.99</v>
       </c>
       <c r="Y15" t="n">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="Z15" t="n">
-        <v>28011</v>
+        <v>109913</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Eicher Motors Ltd</t>
+          <t>Dr Reddys Laboratories Ltd</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1819,86 +1819,86 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>57.1</v>
+        <v>57.2</v>
       </c>
       <c r="F16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G16" t="n">
-        <v>22.17</v>
+        <v>19.74</v>
       </c>
       <c r="H16" t="n">
-        <v>20.21</v>
+        <v>21.36</v>
       </c>
       <c r="I16" t="n">
-        <v>24.2</v>
+        <v>19.91</v>
       </c>
       <c r="J16" t="n">
-        <v>26.18</v>
+        <v>28.32</v>
       </c>
       <c r="K16" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="L16" t="n">
+        <v>51.71</v>
+      </c>
+      <c r="M16" t="n">
+        <v>509</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="O16" t="n">
         <v>0.02</v>
       </c>
-      <c r="L16" t="n">
-        <v>114.71</v>
-      </c>
-      <c r="M16" t="n">
-        <v>890</v>
-      </c>
-      <c r="N16" t="n">
-        <v>5.38</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0.4</v>
-      </c>
       <c r="P16" t="n">
-        <v>23.78</v>
+        <v>13.72</v>
       </c>
       <c r="Q16" t="n">
-        <v>11.04</v>
+        <v>12.64</v>
       </c>
       <c r="R16" t="n">
-        <v>12.68</v>
+        <v>23.39</v>
       </c>
       <c r="S16" t="n">
-        <v>12.51</v>
+        <v>23.84</v>
       </c>
       <c r="T16" t="n">
-        <v>0.93</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="U16" t="n">
-        <v>15.62</v>
+        <v>11.73</v>
       </c>
       <c r="V16" t="n">
-        <v>13.61</v>
+        <v>10.19</v>
       </c>
       <c r="W16" t="n">
-        <v>19.29</v>
+        <v>14.56</v>
       </c>
       <c r="X16" t="n">
-        <v>4.41</v>
+        <v>0.09</v>
       </c>
       <c r="Y16" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="Z16" t="n">
-        <v>16536</v>
+        <v>28011</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pidilite Industries Ltd</t>
+          <t>Eicher Motors Ltd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1907,86 +1907,86 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>55.5</v>
+        <v>57.1</v>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G17" t="n">
-        <v>20.78</v>
+        <v>22.17</v>
       </c>
       <c r="H17" t="n">
-        <v>26.93</v>
+        <v>20.21</v>
       </c>
       <c r="I17" t="n">
-        <v>14.11</v>
+        <v>24.2</v>
       </c>
       <c r="J17" t="n">
-        <v>21.87</v>
+        <v>26.18</v>
       </c>
       <c r="K17" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="L17" t="n">
-        <v>54.33</v>
+        <v>114.71</v>
       </c>
       <c r="M17" t="n">
-        <v>955</v>
+        <v>890</v>
       </c>
       <c r="N17" t="n">
-        <v>7.71</v>
+        <v>5.38</v>
       </c>
       <c r="O17" t="n">
-        <v>0.59</v>
+        <v>0.4</v>
       </c>
       <c r="P17" t="n">
-        <v>19.3</v>
+        <v>23.78</v>
       </c>
       <c r="Q17" t="n">
-        <v>11.84</v>
+        <v>11.04</v>
       </c>
       <c r="R17" t="n">
-        <v>13.49</v>
+        <v>12.68</v>
       </c>
       <c r="S17" t="n">
-        <v>13.56</v>
+        <v>12.51</v>
       </c>
       <c r="T17" t="n">
-        <v>1.56</v>
+        <v>0.93</v>
       </c>
       <c r="U17" t="n">
-        <v>36.12</v>
+        <v>15.62</v>
       </c>
       <c r="V17" t="n">
-        <v>12.3</v>
+        <v>13.61</v>
       </c>
       <c r="W17" t="n">
-        <v>5.36</v>
+        <v>19.29</v>
       </c>
       <c r="X17" t="n">
-        <v>1.01</v>
+        <v>4.41</v>
       </c>
       <c r="Y17" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="Z17" t="n">
-        <v>12383</v>
+        <v>16536</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ICICI Lombard General Insurance Company Ltd</t>
+          <t>Pidilite Industries Ltd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1995,174 +1995,174 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>53</v>
+        <v>55.5</v>
       </c>
       <c r="F18" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G18" t="n">
-        <v>15.72</v>
+        <v>20.78</v>
       </c>
       <c r="H18" t="n">
-        <v>145.23</v>
+        <v>26.93</v>
       </c>
       <c r="I18" t="n">
-        <v>9.369999999999999</v>
+        <v>14.11</v>
       </c>
       <c r="J18" t="n">
-        <v>87.42</v>
+        <v>21.87</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="L18" t="n">
-        <v>160.03</v>
+        <v>54.33</v>
       </c>
       <c r="M18" t="n">
-        <v>486</v>
+        <v>955</v>
       </c>
       <c r="N18" t="n">
-        <v>2.37</v>
+        <v>7.71</v>
       </c>
       <c r="O18" t="n">
-        <v>0.04</v>
+        <v>0.59</v>
       </c>
       <c r="P18" t="n">
-        <v>18.99</v>
+        <v>19.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.91</v>
+        <v>11.84</v>
       </c>
       <c r="R18" t="n">
-        <v>12.84</v>
+        <v>13.49</v>
       </c>
       <c r="S18" t="n">
-        <v>11.14</v>
+        <v>13.56</v>
       </c>
       <c r="T18" t="n">
-        <v>1.25</v>
+        <v>1.56</v>
       </c>
       <c r="U18" t="n">
-        <v>49</v>
+        <v>36.12</v>
       </c>
       <c r="V18" t="n">
-        <v>7.86</v>
+        <v>12.3</v>
       </c>
       <c r="W18" t="n">
-        <v>36.96</v>
+        <v>5.36</v>
       </c>
       <c r="X18" t="n">
-        <v>3.46</v>
+        <v>1.01</v>
       </c>
       <c r="Y18" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="Z18" t="n">
-        <v>20487</v>
+        <v>12383</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Siemens Ltd</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>51.9</v>
+        <v>54.3</v>
       </c>
       <c r="F19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G19" t="n">
-        <v>17.7</v>
+        <v>16.72</v>
       </c>
       <c r="H19" t="n">
-        <v>17.74</v>
+        <v>3.09</v>
       </c>
       <c r="I19" t="n">
-        <v>12.22</v>
+        <v>13.94</v>
       </c>
       <c r="J19" t="n">
-        <v>13.96</v>
+        <v>41.75</v>
       </c>
       <c r="K19" t="n">
-        <v>0.02</v>
+        <v>14.87</v>
       </c>
       <c r="L19" t="n">
-        <v>67.15000000000001</v>
+        <v>1.61</v>
       </c>
       <c r="M19" t="n">
-        <v>1168</v>
+        <v>13296</v>
       </c>
       <c r="N19" t="n">
-        <v>5.25</v>
+        <v>12.03</v>
       </c>
       <c r="O19" t="n">
-        <v>0.1</v>
+        <v>2.68</v>
       </c>
       <c r="P19" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="R19" t="n">
+        <v>85.78</v>
+      </c>
+      <c r="S19" t="n">
+        <v>53.42</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="U19" t="n">
+        <v>36.74</v>
+      </c>
+      <c r="V19" t="n">
+        <v>12.61</v>
+      </c>
+      <c r="W19" t="n">
+        <v>25.23</v>
+      </c>
+      <c r="X19" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="Y19" t="n">
         <v>19</v>
       </c>
-      <c r="Q19" t="n">
-        <v>11.19</v>
-      </c>
-      <c r="R19" t="n">
-        <v>19.85</v>
-      </c>
-      <c r="S19" t="n">
-        <v>19.64</v>
-      </c>
-      <c r="T19" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="U19" t="n">
-        <v>33.32</v>
-      </c>
-      <c r="V19" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="W19" t="n">
-        <v>30.88</v>
-      </c>
-      <c r="X19" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>16</v>
-      </c>
       <c r="Z19" t="n">
-        <v>22240</v>
+        <v>110519</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HAVELLS</t>
+          <t>ICICIGI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Havells India Ltd</t>
+          <t>ICICI Lombard General Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2171,162 +2171,338 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>48.4</v>
+        <v>53</v>
       </c>
       <c r="F20" t="n">
         <v>7</v>
       </c>
       <c r="G20" t="n">
-        <v>17.07</v>
+        <v>15.72</v>
       </c>
       <c r="H20" t="n">
-        <v>19.91</v>
+        <v>145.23</v>
       </c>
       <c r="I20" t="n">
-        <v>6.84</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>10.12</v>
+        <v>87.42</v>
       </c>
       <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>160.03</v>
+      </c>
+      <c r="M20" t="n">
+        <v>486</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="O20" t="n">
         <v>0.04</v>
       </c>
-      <c r="L20" t="n">
-        <v>25.36</v>
-      </c>
-      <c r="M20" t="n">
-        <v>335</v>
-      </c>
-      <c r="N20" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.01</v>
-      </c>
       <c r="P20" t="n">
-        <v>21.14</v>
+        <v>18.99</v>
       </c>
       <c r="Q20" t="n">
-        <v>13.04</v>
+        <v>12.91</v>
       </c>
       <c r="R20" t="n">
-        <v>10.03</v>
+        <v>12.84</v>
       </c>
       <c r="S20" t="n">
-        <v>9</v>
+        <v>11.14</v>
       </c>
       <c r="T20" t="n">
-        <v>1.54</v>
+        <v>1.25</v>
       </c>
       <c r="U20" t="n">
-        <v>45.41</v>
+        <v>49</v>
       </c>
       <c r="V20" t="n">
-        <v>14.08</v>
+        <v>7.86</v>
       </c>
       <c r="W20" t="n">
-        <v>30.73</v>
+        <v>36.96</v>
       </c>
       <c r="X20" t="n">
-        <v>2.6</v>
+        <v>3.46</v>
       </c>
       <c r="Y20" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="Z20" t="n">
-        <v>18590</v>
+        <v>20487</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Siemens Ltd</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="I21" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="J21" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L21" t="n">
+        <v>67.15000000000001</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1168</v>
+      </c>
+      <c r="N21" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="P21" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="R21" t="n">
+        <v>19.85</v>
+      </c>
+      <c r="S21" t="n">
+        <v>19.64</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="U21" t="n">
+        <v>33.32</v>
+      </c>
+      <c r="V21" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="W21" t="n">
+        <v>30.88</v>
+      </c>
+      <c r="X21" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>22240</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HAVELLS</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Havells India Ltd</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7</v>
+      </c>
+      <c r="G22" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="H22" t="n">
+        <v>19.91</v>
+      </c>
+      <c r="I22" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="J22" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L22" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="M22" t="n">
+        <v>335</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P22" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="R22" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="S22" t="n">
+        <v>9</v>
+      </c>
+      <c r="T22" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="U22" t="n">
+        <v>45.41</v>
+      </c>
+      <c r="V22" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="W22" t="n">
+        <v>30.73</v>
+      </c>
+      <c r="X22" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>44</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>18590</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>MARUTI</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Maruti Suzuki India Ltd</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>2024-03</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E23" t="n">
         <v>47.7</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F23" t="n">
         <v>11</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G23" t="n">
         <v>15.75</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H23" t="n">
         <v>15.59</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I23" t="n">
         <v>9.51</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J23" t="n">
         <v>13.13</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K23" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L23" t="n">
         <v>117.91</v>
       </c>
-      <c r="M21" t="n">
+      <c r="M23" t="n">
         <v>4936</v>
       </c>
-      <c r="N21" t="n">
+      <c r="N23" t="n">
         <v>3.48</v>
       </c>
-      <c r="O21" t="n">
+      <c r="O23" t="n">
         <v>0.33</v>
       </c>
-      <c r="P21" t="n">
+      <c r="P23" t="n">
         <v>26.32</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="Q23" t="n">
         <v>10.51</v>
       </c>
-      <c r="R21" t="n">
+      <c r="R23" t="n">
         <v>12.01</v>
       </c>
-      <c r="S21" t="n">
+      <c r="S23" t="n">
         <v>11.14</v>
       </c>
-      <c r="T21" t="n">
+      <c r="T23" t="n">
         <v>1.25</v>
       </c>
-      <c r="U21" t="n">
+      <c r="U23" t="n">
         <v>20.78</v>
       </c>
-      <c r="V21" t="n">
+      <c r="V23" t="n">
         <v>8.26</v>
       </c>
-      <c r="W21" t="n">
+      <c r="W23" t="n">
         <v>29.97</v>
       </c>
-      <c r="X21" t="n">
+      <c r="X23" t="n">
         <v>1.78</v>
       </c>
-      <c r="Y21" t="n">
+      <c r="Y23" t="n">
         <v>29</v>
       </c>
-      <c r="Z21" t="n">
+      <c r="Z23" t="n">
         <v>141858</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G21">
+  <conditionalFormatting sqref="G2:G23">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>15</formula>
     </cfRule>
@@ -2334,7 +2510,7 @@
       <formula>8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H21">
+  <conditionalFormatting sqref="H2:H23">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>15</formula>
     </cfRule>
@@ -2342,7 +2518,7 @@
       <formula>8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I21">
+  <conditionalFormatting sqref="I2:I23">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>10</formula>
     </cfRule>
@@ -2350,7 +2526,7 @@
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K21">
+  <conditionalFormatting sqref="K2:K23">
     <cfRule type="cellIs" priority="7" operator="lessThanOrEqual" dxfId="0">
       <formula>1</formula>
     </cfRule>
@@ -2358,7 +2534,7 @@
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M21">
+  <conditionalFormatting sqref="M2:M23">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2366,7 +2542,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q21">
+  <conditionalFormatting sqref="Q2:Q23">
     <cfRule type="cellIs" priority="11" operator="greaterThanOrEqual" dxfId="0">
       <formula>10</formula>
     </cfRule>
@@ -2374,7 +2550,7 @@
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R21">
+  <conditionalFormatting sqref="R2:R23">
     <cfRule type="cellIs" priority="13" operator="greaterThanOrEqual" dxfId="0">
       <formula>15</formula>
     </cfRule>
@@ -2770,7 +2946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z10"/>
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2996,17 +3172,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Trent Ltd</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3015,86 +3191,86 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>70.8</v>
+        <v>54.3</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>36.31</v>
+        <v>16.72</v>
       </c>
       <c r="H3" t="n">
-        <v>22.33</v>
+        <v>3.09</v>
       </c>
       <c r="I3" t="n">
-        <v>11.94</v>
+        <v>13.94</v>
       </c>
       <c r="J3" t="n">
-        <v>15.93</v>
+        <v>41.75</v>
       </c>
       <c r="K3" t="n">
-        <v>0.43</v>
+        <v>14.87</v>
       </c>
       <c r="L3" t="n">
-        <v>8.039999999999999</v>
+        <v>1.61</v>
       </c>
       <c r="M3" t="n">
-        <v>841</v>
+        <v>13296</v>
       </c>
       <c r="N3" t="n">
-        <v>6.8</v>
+        <v>12.03</v>
       </c>
       <c r="O3" t="n">
-        <v>0.15</v>
+        <v>2.68</v>
       </c>
       <c r="P3" t="n">
-        <v>68.36</v>
+        <v>16.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.31</v>
+        <v>18.18</v>
       </c>
       <c r="R3" t="n">
-        <v>73.11</v>
+        <v>85.78</v>
       </c>
       <c r="S3" t="n">
-        <v>69.52</v>
+        <v>53.42</v>
       </c>
       <c r="T3" t="n">
-        <v>0.91</v>
+        <v>0.98</v>
       </c>
       <c r="U3" t="n">
-        <v>8.65</v>
+        <v>36.74</v>
       </c>
       <c r="V3" t="n">
-        <v>11.82</v>
+        <v>12.61</v>
       </c>
       <c r="W3" t="n">
-        <v>34.65</v>
+        <v>25.23</v>
       </c>
       <c r="X3" t="n">
-        <v>3.46</v>
+        <v>3.81</v>
       </c>
       <c r="Y3" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="Z3" t="n">
-        <v>12375</v>
+        <v>110519</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Adani Enterprises Ltd</t>
+          <t>Bank of Baroda</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3103,81 +3279,81 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>42.1</v>
+        <v>41.7</v>
       </c>
       <c r="F4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G4" t="n">
-        <v>8.529999999999999</v>
+        <v>15.76</v>
       </c>
       <c r="H4" t="n">
-        <v>7.98</v>
+        <v>2.71</v>
       </c>
       <c r="I4" t="n">
-        <v>3.46</v>
+        <v>15.94</v>
       </c>
       <c r="J4" t="n">
-        <v>11.8</v>
+        <v>37.49</v>
       </c>
       <c r="K4" t="n">
-        <v>1.67</v>
+        <v>12.14</v>
       </c>
       <c r="L4" t="n">
-        <v>2.75</v>
+        <v>1.9</v>
       </c>
       <c r="M4" t="n">
-        <v>-8455</v>
+        <v>-7559</v>
       </c>
       <c r="N4" t="n">
-        <v>-8.77</v>
+        <v>-6.39</v>
       </c>
       <c r="O4" t="n">
-        <v>-4.5</v>
+        <v>-1.28</v>
       </c>
       <c r="P4" t="n">
-        <v>34.6</v>
+        <v>16.79</v>
       </c>
       <c r="Q4" t="n">
-        <v>19.02</v>
+        <v>17.48</v>
       </c>
       <c r="R4" t="n">
-        <v>45.81</v>
+        <v>74.51000000000001</v>
       </c>
       <c r="S4" t="n">
-        <v>31.95</v>
+        <v>55.18</v>
       </c>
       <c r="T4" t="n">
-        <v>3.09</v>
+        <v>-0.33</v>
       </c>
       <c r="U4" t="n">
-        <v>58.87</v>
+        <v>16.89</v>
       </c>
       <c r="V4" t="n">
-        <v>10.41</v>
+        <v>4.15</v>
       </c>
       <c r="W4" t="n">
-        <v>33.01</v>
+        <v>24.7</v>
       </c>
       <c r="X4" t="n">
-        <v>0.83</v>
+        <v>2.62</v>
       </c>
       <c r="Y4" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="Z4" t="n">
-        <v>96421</v>
+        <v>118379</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IRCTC</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
+          <t>Trent Ltd</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3191,86 +3367,86 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>77</v>
+        <v>70.8</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>34.4</v>
+        <v>36.31</v>
       </c>
       <c r="H5" t="n">
-        <v>42.83</v>
+        <v>22.33</v>
       </c>
       <c r="I5" t="n">
-        <v>26.02</v>
+        <v>11.94</v>
       </c>
       <c r="J5" t="n">
-        <v>34.33</v>
+        <v>15.93</v>
       </c>
       <c r="K5" t="n">
-        <v>0.02</v>
+        <v>0.43</v>
       </c>
       <c r="L5" t="n">
-        <v>82.73999999999999</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>667</v>
+        <v>841</v>
       </c>
       <c r="N5" t="n">
-        <v>15.62</v>
+        <v>6.8</v>
       </c>
       <c r="O5" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="P5" t="n">
-        <v>76.47</v>
+        <v>68.36</v>
       </c>
       <c r="Q5" t="n">
-        <v>17.96</v>
+        <v>36.31</v>
       </c>
       <c r="R5" t="n">
-        <v>29.17</v>
+        <v>73.11</v>
       </c>
       <c r="S5" t="n">
-        <v>28.47</v>
+        <v>69.52</v>
       </c>
       <c r="T5" t="n">
-        <v>0.79</v>
+        <v>0.91</v>
       </c>
       <c r="U5" t="n">
-        <v>60.44</v>
+        <v>8.65</v>
       </c>
       <c r="V5" t="n">
-        <v>5.74</v>
+        <v>11.82</v>
       </c>
       <c r="W5" t="n">
-        <v>32.47</v>
+        <v>34.65</v>
       </c>
       <c r="X5" t="n">
-        <v>1.08</v>
+        <v>3.46</v>
       </c>
       <c r="Y5" t="n">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="Z5" t="n">
-        <v>4270</v>
+        <v>12375</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LTIM</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LTIMindtree Ltd</t>
+          <t>ICICI Bank Ltd</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3279,86 +3455,86 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63.5</v>
+        <v>61.8</v>
       </c>
       <c r="F6" t="n">
         <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>22.9</v>
+        <v>17.99</v>
       </c>
       <c r="H6" t="n">
-        <v>25.21</v>
+        <v>5.12</v>
       </c>
       <c r="I6" t="n">
-        <v>12.91</v>
+        <v>28.89</v>
       </c>
       <c r="J6" t="n">
-        <v>17.98</v>
+        <v>62.41</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1</v>
+        <v>6.45</v>
       </c>
       <c r="L6" t="n">
-        <v>31.93</v>
+        <v>1.3</v>
       </c>
       <c r="M6" t="n">
-        <v>1752</v>
+        <v>12547</v>
       </c>
       <c r="N6" t="n">
-        <v>4.93</v>
+        <v>7.87</v>
       </c>
       <c r="O6" t="n">
-        <v>0.13</v>
+        <v>0.95</v>
       </c>
       <c r="P6" t="n">
-        <v>42.13</v>
+        <v>21.4</v>
       </c>
       <c r="Q6" t="n">
-        <v>30.33</v>
+        <v>17.25</v>
       </c>
       <c r="R6" t="n">
-        <v>24.78</v>
+        <v>51.95</v>
       </c>
       <c r="S6" t="n">
-        <v>12.24</v>
+        <v>55.18</v>
       </c>
       <c r="T6" t="n">
-        <v>1.24</v>
+        <v>3.41</v>
       </c>
       <c r="U6" t="n">
-        <v>64.52</v>
+        <v>25.76</v>
       </c>
       <c r="V6" t="n">
-        <v>2.38</v>
+        <v>6.2</v>
       </c>
       <c r="W6" t="n">
-        <v>18.9</v>
+        <v>38.28</v>
       </c>
       <c r="X6" t="n">
-        <v>4.43</v>
+        <v>3.43</v>
       </c>
       <c r="Y6" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="Z6" t="n">
-        <v>35517</v>
+        <v>159516</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ATGL</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Adani Total Gas Ltd</t>
+          <t>Adani Enterprises Ltd</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3367,86 +3543,86 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>61.1</v>
+        <v>42.1</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>18.66</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>18.42</v>
+        <v>7.98</v>
       </c>
       <c r="I7" t="n">
-        <v>14.93</v>
+        <v>3.46</v>
       </c>
       <c r="J7" t="n">
-        <v>24.67</v>
+        <v>11.8</v>
       </c>
       <c r="K7" t="n">
-        <v>0.43</v>
+        <v>1.67</v>
       </c>
       <c r="L7" t="n">
-        <v>10.5</v>
+        <v>2.75</v>
       </c>
       <c r="M7" t="n">
-        <v>203</v>
+        <v>-8455</v>
       </c>
       <c r="N7" t="n">
-        <v>4.54</v>
+        <v>-8.77</v>
       </c>
       <c r="O7" t="n">
-        <v>0.01</v>
+        <v>-4.5</v>
       </c>
       <c r="P7" t="n">
-        <v>38.18</v>
+        <v>34.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>21.09</v>
+        <v>19.02</v>
       </c>
       <c r="R7" t="n">
-        <v>23.88</v>
+        <v>45.81</v>
       </c>
       <c r="S7" t="n">
-        <v>24.57</v>
+        <v>31.95</v>
       </c>
       <c r="T7" t="n">
-        <v>1.43</v>
+        <v>3.09</v>
       </c>
       <c r="U7" t="n">
-        <v>56.96</v>
+        <v>58.87</v>
       </c>
       <c r="V7" t="n">
-        <v>5.76</v>
+        <v>10.41</v>
       </c>
       <c r="W7" t="n">
-        <v>28.93</v>
+        <v>33.01</v>
       </c>
       <c r="X7" t="n">
-        <v>0.51</v>
+        <v>0.83</v>
       </c>
       <c r="Y7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Z7" t="n">
-        <v>4475</v>
+        <v>96421</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DMART</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Avenue Supermarts Ltd</t>
+          <t>Bajaj Finance Ltd</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3455,86 +3631,86 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>53.7</v>
+        <v>39.9</v>
       </c>
       <c r="F8" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G8" t="n">
-        <v>13.56</v>
+        <v>18.84</v>
       </c>
       <c r="H8" t="n">
-        <v>17.5</v>
+        <v>4.17</v>
       </c>
       <c r="I8" t="n">
-        <v>4.99</v>
+        <v>26.29</v>
       </c>
       <c r="J8" t="n">
-        <v>8.08</v>
+        <v>29.29</v>
       </c>
       <c r="K8" t="n">
-        <v>0.03</v>
+        <v>3.82</v>
       </c>
       <c r="L8" t="n">
-        <v>73.29000000000001</v>
+        <v>2689.17</v>
       </c>
       <c r="M8" t="n">
-        <v>278</v>
+        <v>-79931</v>
       </c>
       <c r="N8" t="n">
-        <v>0.55</v>
+        <v>-145.4</v>
       </c>
       <c r="O8" t="n">
-        <v>0.01</v>
+        <v>-3.23</v>
       </c>
       <c r="P8" t="n">
-        <v>28.13</v>
+        <v>27.26</v>
       </c>
       <c r="Q8" t="n">
-        <v>20.48</v>
+        <v>24.35</v>
       </c>
       <c r="R8" t="n">
-        <v>22.97</v>
+        <v>29.32</v>
       </c>
       <c r="S8" t="n">
-        <v>22.74</v>
+        <v>27.56</v>
       </c>
       <c r="T8" t="n">
-        <v>1.08</v>
+        <v>-5.03</v>
       </c>
       <c r="U8" t="n">
-        <v>72.53</v>
+        <v>69.2</v>
       </c>
       <c r="V8" t="n">
-        <v>11.71</v>
+        <v>4.11</v>
       </c>
       <c r="W8" t="n">
-        <v>36.84</v>
+        <v>15.96</v>
       </c>
       <c r="X8" t="n">
-        <v>1.94</v>
+        <v>0.27</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="Z8" t="n">
-        <v>50789</v>
+        <v>54972</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>IRCTC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tata Consumer Products Ltd</t>
+          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3543,162 +3719,1042 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>49</v>
+        <v>77</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>7.57</v>
+        <v>34.4</v>
       </c>
       <c r="H9" t="n">
-        <v>9.76</v>
+        <v>42.83</v>
       </c>
       <c r="I9" t="n">
-        <v>7.99</v>
+        <v>26.02</v>
       </c>
       <c r="J9" t="n">
-        <v>15.02</v>
+        <v>34.33</v>
       </c>
       <c r="K9" t="n">
-        <v>0.22</v>
+        <v>0.02</v>
       </c>
       <c r="L9" t="n">
-        <v>25.32</v>
+        <v>82.73999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>26</v>
+        <v>667</v>
       </c>
       <c r="N9" t="n">
-        <v>0.17</v>
+        <v>15.62</v>
       </c>
       <c r="O9" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="P9" t="n">
-        <v>9.44</v>
+        <v>76.47</v>
       </c>
       <c r="Q9" t="n">
-        <v>15.96</v>
+        <v>17.96</v>
       </c>
       <c r="R9" t="n">
-        <v>21.6</v>
+        <v>29.17</v>
       </c>
       <c r="S9" t="n">
-        <v>14.87</v>
+        <v>28.47</v>
       </c>
       <c r="T9" t="n">
-        <v>1.59</v>
+        <v>0.79</v>
       </c>
       <c r="U9" t="n">
-        <v>54.79</v>
+        <v>60.44</v>
       </c>
       <c r="V9" t="n">
-        <v>7.14</v>
+        <v>5.74</v>
       </c>
       <c r="W9" t="n">
-        <v>24.84</v>
+        <v>32.47</v>
       </c>
       <c r="X9" t="n">
-        <v>1.87</v>
+        <v>1.08</v>
       </c>
       <c r="Y9" t="n">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="Z9" t="n">
-        <v>15206</v>
+        <v>4270</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>LTIM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LTIMindtree Ltd</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="H10" t="n">
+        <v>25.21</v>
+      </c>
+      <c r="I10" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="J10" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>31.93</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1752</v>
+      </c>
+      <c r="N10" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="P10" t="n">
+        <v>42.13</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>30.33</v>
+      </c>
+      <c r="R10" t="n">
+        <v>24.78</v>
+      </c>
+      <c r="S10" t="n">
+        <v>12.24</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="U10" t="n">
+        <v>64.52</v>
+      </c>
+      <c r="V10" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="W10" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="X10" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>42</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>35517</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ATGL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Adani Total Gas Ltd</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18.66</v>
+      </c>
+      <c r="H11" t="n">
+        <v>18.42</v>
+      </c>
+      <c r="I11" t="n">
+        <v>14.93</v>
+      </c>
+      <c r="J11" t="n">
+        <v>24.67</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="L11" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="M11" t="n">
+        <v>203</v>
+      </c>
+      <c r="N11" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P11" t="n">
+        <v>38.18</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>21.09</v>
+      </c>
+      <c r="R11" t="n">
+        <v>23.88</v>
+      </c>
+      <c r="S11" t="n">
+        <v>24.57</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="U11" t="n">
+        <v>56.96</v>
+      </c>
+      <c r="V11" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="W11" t="n">
+        <v>28.93</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>4475</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HDFC Bank Ltd</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="F12" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" t="n">
+        <v>14.34</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I12" t="n">
+        <v>23.07</v>
+      </c>
+      <c r="J12" t="n">
+        <v>61.41</v>
+      </c>
+      <c r="K12" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="M12" t="n">
+        <v>35669</v>
+      </c>
+      <c r="N12" t="n">
+        <v>12.58</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="P12" t="n">
+        <v>30.19</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="R12" t="n">
+        <v>23.87</v>
+      </c>
+      <c r="S12" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="U12" t="n">
+        <v>49.42</v>
+      </c>
+      <c r="V12" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="W12" t="n">
+        <v>22.54</v>
+      </c>
+      <c r="X12" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>283649</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bajaj Finserv Ltd</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="F13" t="n">
+        <v>18</v>
+      </c>
+      <c r="G13" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="H13" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="I13" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="J13" t="n">
+        <v>37.04</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M13" t="n">
+        <v>-79634</v>
+      </c>
+      <c r="N13" t="n">
+        <v>-72.14</v>
+      </c>
+      <c r="O13" t="n">
+        <v>-4.18</v>
+      </c>
+      <c r="P13" t="n">
+        <v>22.13</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="R13" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="S13" t="n">
+        <v>20.59</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="U13" t="n">
+        <v>15.07</v>
+      </c>
+      <c r="V13" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="W13" t="n">
+        <v>39.72</v>
+      </c>
+      <c r="X13" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>110382</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Shriram Finance Ltd</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="F14" t="n">
+        <v>23</v>
+      </c>
+      <c r="G14" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="I14" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="J14" t="n">
+        <v>28.92</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="M14" t="n">
+        <v>-31359</v>
+      </c>
+      <c r="N14" t="n">
+        <v>-86.18000000000001</v>
+      </c>
+      <c r="O14" t="n">
+        <v>-3.61</v>
+      </c>
+      <c r="P14" t="n">
+        <v>27.83</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>18.56</v>
+      </c>
+      <c r="R14" t="n">
+        <v>23.49</v>
+      </c>
+      <c r="S14" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="U14" t="n">
+        <v>68.53</v>
+      </c>
+      <c r="V14" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="W14" t="n">
+        <v>28.82</v>
+      </c>
+      <c r="X14" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>36388</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>17</v>
+      </c>
+      <c r="G15" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="I15" t="n">
+        <v>17.85</v>
+      </c>
+      <c r="J15" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>6.86</v>
+      </c>
+      <c r="L15" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-38538</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-201.11</v>
+      </c>
+      <c r="O15" t="n">
+        <v>-3.97</v>
+      </c>
+      <c r="P15" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>21.94</v>
+      </c>
+      <c r="R15" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="S15" t="n">
+        <v>22.28</v>
+      </c>
+      <c r="T15" t="n">
+        <v>-10.43</v>
+      </c>
+      <c r="U15" t="n">
+        <v>16.79</v>
+      </c>
+      <c r="V15" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="W15" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="X15" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>19163</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Indian Railway Finance Corporation Ltd</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="H16" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="I16" t="n">
+        <v>24.06</v>
+      </c>
+      <c r="J16" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="K16" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="M16" t="n">
+        <v>7906</v>
+      </c>
+      <c r="N16" t="n">
+        <v>29.67</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P16" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>19.07</v>
+      </c>
+      <c r="R16" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="S16" t="n">
+        <v>20.11</v>
+      </c>
+      <c r="T16" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="U16" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="V16" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="W16" t="n">
+        <v>16.66</v>
+      </c>
+      <c r="X16" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>31</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>26645</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Avenue Supermarts Ltd</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="H17" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L17" t="n">
+        <v>73.29000000000001</v>
+      </c>
+      <c r="M17" t="n">
+        <v>278</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P17" t="n">
+        <v>28.13</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="R17" t="n">
+        <v>22.97</v>
+      </c>
+      <c r="S17" t="n">
+        <v>22.74</v>
+      </c>
+      <c r="T17" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="U17" t="n">
+        <v>72.53</v>
+      </c>
+      <c r="V17" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="W17" t="n">
+        <v>36.84</v>
+      </c>
+      <c r="X17" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>50789</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>INDUSINDBK</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IndusInd Bank Ltd</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>22</v>
+      </c>
+      <c r="G18" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="H18" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="I18" t="n">
+        <v>19.56</v>
+      </c>
+      <c r="J18" t="n">
+        <v>38.55</v>
+      </c>
+      <c r="K18" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="M18" t="n">
+        <v>-17468</v>
+      </c>
+      <c r="N18" t="n">
+        <v>-38.18</v>
+      </c>
+      <c r="O18" t="n">
+        <v>-0.97</v>
+      </c>
+      <c r="P18" t="n">
+        <v>16.41</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="R18" t="n">
+        <v>22.08</v>
+      </c>
+      <c r="S18" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="T18" t="n">
+        <v>-1.88</v>
+      </c>
+      <c r="U18" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="W18" t="n">
+        <v>28.79</v>
+      </c>
+      <c r="X18" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>45748</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Tata Consumer Products Ltd</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>49</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="H19" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="I19" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="J19" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="L19" t="n">
+        <v>25.32</v>
+      </c>
+      <c r="M19" t="n">
+        <v>26</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P19" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>15.96</v>
+      </c>
+      <c r="R19" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="S19" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="T19" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="U19" t="n">
+        <v>54.79</v>
+      </c>
+      <c r="V19" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="W19" t="n">
+        <v>24.84</v>
+      </c>
+      <c r="X19" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>64</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>15206</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>TITAN</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Titan Company Ltd</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>2024-03</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E20" t="n">
         <v>58.5</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F20" t="n">
         <v>4</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G20" t="n">
         <v>37.22</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H20" t="n">
         <v>18.89</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I20" t="n">
         <v>6.84</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J20" t="n">
         <v>10.36</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K20" t="n">
         <v>1.65</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L20" t="n">
         <v>9.41</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M20" t="n">
         <v>1506</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N20" t="n">
         <v>2.95</v>
       </c>
-      <c r="O10" t="n">
+      <c r="O20" t="n">
         <v>0.08</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P20" t="n">
         <v>33.14</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q20" t="n">
         <v>20.9</v>
       </c>
-      <c r="R10" t="n">
+      <c r="R20" t="n">
         <v>20.27</v>
       </c>
-      <c r="S10" t="n">
+      <c r="S20" t="n">
         <v>19.51</v>
       </c>
-      <c r="T10" t="n">
+      <c r="T20" t="n">
         <v>0.48</v>
       </c>
-      <c r="U10" t="n">
+      <c r="U20" t="n">
         <v>10.13</v>
       </c>
-      <c r="V10" t="n">
+      <c r="V20" t="n">
         <v>10.51</v>
       </c>
-      <c r="W10" t="n">
+      <c r="W20" t="n">
         <v>21</v>
       </c>
-      <c r="X10" t="n">
+      <c r="X20" t="n">
         <v>3.1</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Y20" t="n">
         <v>28</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="Z20" t="n">
         <v>51084</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G10">
+  <conditionalFormatting sqref="G2:G20">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>15</formula>
     </cfRule>
@@ -3706,7 +4762,7 @@
       <formula>8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H10">
+  <conditionalFormatting sqref="H2:H20">
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>15</formula>
     </cfRule>
@@ -3714,7 +4770,7 @@
       <formula>8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I10">
+  <conditionalFormatting sqref="I2:I20">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>10</formula>
     </cfRule>
@@ -3722,7 +4778,7 @@
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K10">
+  <conditionalFormatting sqref="K2:K20">
     <cfRule type="cellIs" priority="7" operator="lessThanOrEqual" dxfId="0">
       <formula>1</formula>
     </cfRule>
@@ -3730,7 +4786,7 @@
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M10">
+  <conditionalFormatting sqref="M2:M20">
     <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3738,7 +4794,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q10">
+  <conditionalFormatting sqref="Q2:Q20">
     <cfRule type="cellIs" priority="11" operator="greaterThanOrEqual" dxfId="0">
       <formula>10</formula>
     </cfRule>
@@ -3746,7 +4802,7 @@
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R10">
+  <conditionalFormatting sqref="R2:R20">
     <cfRule type="cellIs" priority="13" operator="greaterThanOrEqual" dxfId="0">
       <formula>15</formula>
     </cfRule>

</xml_diff>